<commit_message>
testing 151 websites till today
</commit_message>
<xml_diff>
--- a/shieldscope_scan_report.xlsx
+++ b/shieldscope_scan_report.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3491,6 +3491,2529 @@
         </is>
       </c>
     </row>
+    <row r="83" ht="54" customHeight="1">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:42:17 UTC</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="90" customHeight="1">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>https://www.microsoft.com</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:43:18 UTC</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="24" customHeight="1">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>https://www.apple.com</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:43:58 UTC</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="24" customHeight="1">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>https://www.apple.com</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:50:33 UTC</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="54" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.samsung.com</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:51:03 UTC</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="90" customHeight="1">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sony.com</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:51:21 UTC</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="90" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lg.com</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:51:51 UTC</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="24" customHeight="1">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lenovo.com</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:52:19 UTC</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>[HIGH] Origin check bypass using lookalike origin 'https://evil-www.lenovo.com'</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="24" customHeight="1">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asus.com</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:52:59 UTC</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="24" customHeight="1">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>https://www.acer.com</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:53:50 UTC</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="54" customHeight="1">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nvidia.com</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:54:18 UTC</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>[LOW] Access-Control-Allow-Origin is set to '*'</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="24" customHeight="1">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amd.com</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:54:52 UTC</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="54" customHeight="1">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>https://www.qualcomm.com</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:55:22 UTC</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>[CRITICAL] /.env
+[CRITICAL] /.env.production
+[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="90" customHeight="1">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sap.com</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:55:45 UTC</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>[HIGH] Origin check bypass using lookalike origin 'https://evil-www.sap.com'</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="24" customHeight="1">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>https://www.salesforce.com</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:56:12 UTC</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="24" customHeight="1">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>https://www.intuit.com</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:56:29 UTC</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="36" customHeight="1">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>https://www.autodesk.com</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Technology &amp; SaaS</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:56:47 UTC</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="54" customHeight="1">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:57:12 UTC</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="54" customHeight="1">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>https://www.costco.com</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:59:14 UTC</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="90" customHeight="1">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>https://www.homedepot.com</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:59:45 UTC</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="72" customHeight="1">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>https://www.macys.com</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:00:40 UTC</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>[HIGH] Origin check bypass using lookalike origin 'https://evil-www.macys.com'</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="72" customHeight="1">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nike.com</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:02:21 UTC</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="54" customHeight="1">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>https://www.puma.com</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:03:17 UTC</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>[LOW] Access-Control-Allow-Origin is set to '*'</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="54" customHeight="1">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>https://www.uniqlo.com</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:04:36 UTC</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="90" customHeight="1">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hm.com</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:04:52 UTC</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="72" customHeight="1">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>https://www.zara.com</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:05:10 UTC</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G108" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="54" customHeight="1">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>https://www.levi.com</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:05:27 UTC</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="90" customHeight="1">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>https://www.underarmour.com</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:06:27 UTC</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="24" customHeight="1">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lululemon.com</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:07:32 UTC</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="24" customHeight="1">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ubereats.com</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:08:08 UTC</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G112" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="24" customHeight="1">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>https://www.doordash.com</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:08:29 UTC</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F113" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G113" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="24" customHeight="1">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>https://www.grubhub.com</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:09:04 UTC</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F114" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G114" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="24" customHeight="1">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kroger.com</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:15:37 UTC</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F115" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="24" customHeight="1">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wholefoodsmarket.com</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:17:55 UTC</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F116" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="24" customHeight="1">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dominos.com</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:18:20 UTC</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F117" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G117" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="24" customHeight="1">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pizzahut.com</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:19:05 UTC</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G118" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="90" customHeight="1">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kfc.com</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:19:32 UTC</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F119" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="24" customHeight="1">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mcdonalds.com</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:20:36 UTC</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="36" customHeight="1">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>https://www.starbucks.com</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:21:14 UTC</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>Missing: X-Frame-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G121" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="24" customHeight="1">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>https://www.subway.com</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D122" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:21:45 UTC</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="36" customHeight="1">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>https://www.coca-cola.com</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:22:07 UTC</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>Missing: X-Frame-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="inlineStr">
+        <is>
+          <t>[HIGH] Origin check bypass using lookalike origin 'https://evil-www.coca-cola.com'</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="72" customHeight="1">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pepsi.com</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:22:26 UTC</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="36" customHeight="1">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nestle.com</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:22:50 UTC</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="90" customHeight="1">
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>https://www.unilever.com</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:23:21 UTC</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="24" customHeight="1">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pg.com</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:24:05 UTC</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F127" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="90" customHeight="1">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jnj.com</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D128" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:24:30 UTC</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="24" customHeight="1">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pfizer.com</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:24:54 UTC</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="36" customHeight="1">
+      <c r="A130" s="4" t="inlineStr">
+        <is>
+          <t>https://www.roche.com</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:26:04 UTC</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>Missing: X-Frame-Options
+Missing: X-Content-Type-Options</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="36" customHeight="1">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>https://www.novartis.com</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:26:55 UTC</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G131" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="24" customHeight="1">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gsk.com</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D132" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:27:46 UTC</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F132" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G132" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="24" customHeight="1">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>https://www.merck.com</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:28:05 UTC</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G133" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="90" customHeight="1">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bayer.com</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:28:42 UTC</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F134" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="24" customHeight="1">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sanofi.com</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:29:03 UTC</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G135" s="4" t="inlineStr">
+        <is>
+          <t>[LOW] Access-Control-Allow-Origin is set to '*'</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="24" customHeight="1">
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>https://www.who.int</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D136" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:29:30 UTC</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="inlineStr">
+        <is>
+          <t>[LOW] Access-Control-Allow-Origin is set to '*'</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="72" customHeight="1">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:30:05 UTC</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F137" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G137" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="24" customHeight="1">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nih.gov</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:30:48 UTC</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G138" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="72" customHeight="1">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>https://www.webmd.com</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:32:03 UTC</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F139" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G139" s="4" t="inlineStr">
+        <is>
+          <t>[LOW] Access-Control-Allow-Origin is set to '*'</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="72" customHeight="1">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>https://www.healthline.com</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="D140" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:32:32 UTC</t>
+        </is>
+      </c>
+      <c r="E140" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F140" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G140" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="90" customHeight="1">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mayoclinic.org</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:33:17 UTC</t>
+        </is>
+      </c>
+      <c r="E141" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F141" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G141" s="4" t="inlineStr">
+        <is>
+          <t>[MEDIUM] Arbitrary origin reflected in Access-Control-Allow-Origin
+[HIGH] Origin check bypass using lookalike origin 'https://www.mayoclinic.org.evil-attacker-test.com'
+[HIGH] Origin check bypass using lookalike origin 'https://evil-www.mayoclinic.org'
+[MEDIUM] Explicitly accepting 'null' origin in CORS policy
+[MEDIUM] Dynamic origin reflection without specifying Vary: Origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="36" customHeight="1">
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>https://www.clevelandclinic.org</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:34:16 UTC</t>
+        </is>
+      </c>
+      <c r="E142" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F142" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G142" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="90" customHeight="1">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>https://www.harvard.edu</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 14:35:09 UTC</t>
+        </is>
+      </c>
+      <c r="E143" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F143" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G143" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="36" customHeight="1">
+      <c r="A144" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mit.edu</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D144" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:48:55 UTC</t>
+        </is>
+      </c>
+      <c r="E144" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F144" s="4" t="inlineStr">
+        <is>
+          <t>Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G144" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="24" customHeight="1">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>https://www.stanford.edu</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:50:41 UTC</t>
+        </is>
+      </c>
+      <c r="E145" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F145" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G145" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="54" customHeight="1">
+      <c r="A146" s="4" t="inlineStr">
+        <is>
+          <t>https://www.berkeley.edu</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:51:19 UTC</t>
+        </is>
+      </c>
+      <c r="E146" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F146" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: X-Content-Type-Options</t>
+        </is>
+      </c>
+      <c r="G146" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="54" customHeight="1">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>https://www.princeton.edu</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:51:47 UTC</t>
+        </is>
+      </c>
+      <c r="E147" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F147" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Strict-Transport-Security
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G147" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="36" customHeight="1">
+      <c r="A148" s="4" t="inlineStr">
+        <is>
+          <t>https://www.yale.edu</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:52:18 UTC</t>
+        </is>
+      </c>
+      <c r="E148" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F148" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G148" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="24" customHeight="1">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cornell.edu</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:52:42 UTC</t>
+        </is>
+      </c>
+      <c r="E149" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F149" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G149" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="24" customHeight="1">
+      <c r="A150" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cornell.edu</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D150" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:53:06 UTC</t>
+        </is>
+      </c>
+      <c r="E150" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F150" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G150" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="24" customHeight="1">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ox.ac.uk</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10 17:53:26 UTC</t>
+        </is>
+      </c>
+      <c r="E151" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F151" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G151" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
testing IT industries  websites
</commit_message>
<xml_diff>
--- a/shieldscope_scan_report.xlsx
+++ b/shieldscope_scan_report.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G188"/>
+  <dimension ref="A1:G195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -7348,6 +7348,259 @@
         </is>
       </c>
     </row>
+    <row r="189" ht="24" customHeight="1">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>https://www.accenture.com</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:57:54 UTC</t>
+        </is>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G189" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="54" customHeight="1">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>https://www.tcs.com</t>
+        </is>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D190" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:58:13 UTC</t>
+        </is>
+      </c>
+      <c r="E190" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F190" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G190" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="72" customHeight="1">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t>https://www.infosys.com</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:58:37 UTC</t>
+        </is>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G191" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="72" customHeight="1">
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t>https://www.infosys.com</t>
+        </is>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D192" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:58:59 UTC</t>
+        </is>
+      </c>
+      <c r="E192" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F192" s="4" t="inlineStr">
+        <is>
+          <t>Missing: Content-Security-Policy
+Missing: X-Frame-Options
+Missing: X-Content-Type-Options
+Missing: Referrer-Policy</t>
+        </is>
+      </c>
+      <c r="G192" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="24" customHeight="1">
+      <c r="A193" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wipro.com</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:59:25 UTC</t>
+        </is>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G193" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="24" customHeight="1">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hcltech.com</t>
+        </is>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D194" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:59:48 UTC</t>
+        </is>
+      </c>
+      <c r="E194" s="4" t="inlineStr">
+        <is>
+          <t>None (Secure)</t>
+        </is>
+      </c>
+      <c r="F194" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G194" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="24" customHeight="1">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>https://www.capgemini.com</t>
+        </is>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D195" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 14:00:17 UTC</t>
+        </is>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] /.well-known/security.txt</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="inlineStr">
+        <is>
+          <t>None (All Secure)</t>
+        </is>
+      </c>
+      <c r="G195" s="4" t="inlineStr">
+        <is>
+          <t>[INFO] No CORS misconfiguration detected</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>